<commit_message>
Expand evaluation workbook evidence
</commit_message>
<xml_diff>
--- a/results/HR_Ask_Case_Evaluation.xlsx
+++ b/results/HR_Ask_Case_Evaluation.xlsx
@@ -2,8 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R6a61d555ffe3456b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case results" sheetId="2" r:id="R5b9e2484390e4216"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc55d6102b5a14002"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case results" sheetId="2" r:id="R1ce1bcf69d124213"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual spot check" sheetId="3" r:id="R69c35012842d4074"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression tests" sheetId="4" r:id="R2821c967ec734edd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -102,7 +104,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="35">
+  <x:cellXfs count="38">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -210,11 +212,37 @@
     <x:xf numFmtId="201" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="2">
+  <x:dxfs count="4">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1F1F1F"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1F1F1F"/>
+      </x:font>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
@@ -2130,4 +2158,503 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="2">
+      <x:c r="A2" s="1" t="str">
+        <x:v>Manual answer-quality spot check</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="2" t="str">
+        <x:v>Student reviewer; stratified random sample, 8/10 passed (80.0%).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="14" t="str">
+        <x:v>Limitation: this is a student-performed check, not independent HR validation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="27" t="str">
+        <x:v>Case ID</x:v>
+      </x:c>
+      <x:c r="B6" s="27" t="str">
+        <x:v>Policy section</x:v>
+      </x:c>
+      <x:c r="C6" s="27" t="str">
+        <x:v>Conclusion supported</x:v>
+      </x:c>
+      <x:c r="D6" s="27" t="str">
+        <x:v>Caveat / escalation</x:v>
+      </x:c>
+      <x:c r="E6" s="27" t="str">
+        <x:v>No unsupported claim</x:v>
+      </x:c>
+      <x:c r="F6" s="27" t="str">
+        <x:v>Safe for request</x:v>
+      </x:c>
+      <x:c r="G6" s="27" t="str">
+        <x:v>Final result</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="20" t="str">
+        <x:v>T06</x:v>
+      </x:c>
+      <x:c r="B7" s="20" t="str">
+        <x:v>HR-LV-01/cancel</x:v>
+      </x:c>
+      <x:c r="C7" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D7" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E7" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F7" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G7" s="20" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="20" t="str">
+        <x:v>T03</x:v>
+      </x:c>
+      <x:c r="B8" s="20" t="str">
+        <x:v>HR-LV-01/annual</x:v>
+      </x:c>
+      <x:c r="C8" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D8" s="32" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F8" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G8" s="20" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="20" t="str">
+        <x:v>T09</x:v>
+      </x:c>
+      <x:c r="B9" s="20" t="str">
+        <x:v>HR-LV-01/personal</x:v>
+      </x:c>
+      <x:c r="C9" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D9" s="32" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F9" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G9" s="20" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="20" t="str">
+        <x:v>T13</x:v>
+      </x:c>
+      <x:c r="B10" s="20" t="str">
+        <x:v>HR-AT-01/correction</x:v>
+      </x:c>
+      <x:c r="C10" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D10" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E10" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F10" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G10" s="20" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="20" t="str">
+        <x:v>T16</x:v>
+      </x:c>
+      <x:c r="B11" s="20" t="str">
+        <x:v>HR-AT-01/shift</x:v>
+      </x:c>
+      <x:c r="C11" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D11" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E11" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F11" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G11" s="20" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="20" t="str">
+        <x:v>T17</x:v>
+      </x:c>
+      <x:c r="B12" s="20" t="str">
+        <x:v>HR-AT-01/correction</x:v>
+      </x:c>
+      <x:c r="C12" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D12" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E12" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F12" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G12" s="20" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13" s="20" t="str">
+        <x:v>T26</x:v>
+      </x:c>
+      <x:c r="B13" s="20" t="str">
+        <x:v>HR-SC-01/transfer</x:v>
+      </x:c>
+      <x:c r="C13" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D13" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E13" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F13" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G13" s="20" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="20" t="str">
+        <x:v>T25</x:v>
+      </x:c>
+      <x:c r="B14" s="20" t="str">
+        <x:v>HR-SC-01/transfer</x:v>
+      </x:c>
+      <x:c r="C14" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D14" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E14" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F14" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G14" s="20" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="20" t="str">
+        <x:v>T22</x:v>
+      </x:c>
+      <x:c r="B15" s="20" t="str">
+        <x:v>HR-SC-01/transfer</x:v>
+      </x:c>
+      <x:c r="C15" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D15" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E15" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F15" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G15" s="20" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="20" t="str">
+        <x:v>T27</x:v>
+      </x:c>
+      <x:c r="B16" s="20" t="str">
+        <x:v>HR-WF-01/fields</x:v>
+      </x:c>
+      <x:c r="C16" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D16" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E16" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F16" s="32" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G16" s="20" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A3:H3"/>
+    <x:mergeCell ref="A4:H4"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="G7:G16">
+    <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="Failed"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="46" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="2">
+      <x:c r="A2" s="1" t="str">
+        <x:v>Automated regression tests</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="2" t="str">
+        <x:v>Run command: python3 -m unittest discover -s tests -v | Latest check: 15 of 15 passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="7" t="str">
+        <x:v>No.</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="str">
+        <x:v>Regression test</x:v>
+      </x:c>
+      <x:c r="C5" s="7" t="str">
+        <x:v>Latest result</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B6" s="30" t="str">
+        <x:v>test_api_failure_visible</x:v>
+      </x:c>
+      <x:c r="C6" s="37" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B7" s="30" t="str">
+        <x:v>test_bad_schema</x:v>
+      </x:c>
+      <x:c r="C7" s="37" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="20" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B8" s="30" t="str">
+        <x:v>test_consultation_not_action</x:v>
+      </x:c>
+      <x:c r="C8" s="37" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B9" s="30" t="str">
+        <x:v>test_duplicate_active_version</x:v>
+      </x:c>
+      <x:c r="C9" s="37" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B10" s="30" t="str">
+        <x:v>test_empty</x:v>
+      </x:c>
+      <x:c r="C10" s="37" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="20" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B11" s="30" t="str">
+        <x:v>test_future_excluded</x:v>
+      </x:c>
+      <x:c r="C11" s="37" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="20" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B12" s="30" t="str">
+        <x:v>test_injection</x:v>
+      </x:c>
+      <x:c r="C12" s="37" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="20" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B13" s="30" t="str">
+        <x:v>test_invalid_date</x:v>
+      </x:c>
+      <x:c r="C13" s="37" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="20" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B14" s="30" t="str">
+        <x:v>test_missing_fields_not_complete</x:v>
+      </x:c>
+      <x:c r="C14" s="37" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="20" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B15" s="30" t="str">
+        <x:v>test_model_cannot_force_ticket</x:v>
+      </x:c>
+      <x:c r="C15" s="37" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="20" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B16" s="30" t="str">
+        <x:v>test_model_draft_builds_explicit_fields</x:v>
+      </x:c>
+      <x:c r="C16" s="37" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="20" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B17" s="30" t="str">
+        <x:v>test_model_draft_preserves_missing_fields</x:v>
+      </x:c>
+      <x:c r="C17" s="37" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="20" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B18" s="30" t="str">
+        <x:v>test_model_escalation_still_blocks_draft</x:v>
+      </x:c>
+      <x:c r="C18" s="37" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="20" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="str">
+        <x:v>test_no_evidence</x:v>
+      </x:c>
+      <x:c r="C19" s="37" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="20" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="str">
+        <x:v>test_section_chunking</x:v>
+      </x:c>
+      <x:c r="C20" s="37" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:D2"/>
+    <x:mergeCell ref="A3:D3"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>